<commit_message>
Definir metricas y storytelling para parcial Power BI
</commit_message>
<xml_diff>
--- a/clase_s1/datasets_powerbi_parcial/01_ventas_retail_powerbi.xlsx
+++ b/clase_s1/datasets_powerbi_parcial/01_ventas_retail_powerbi.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ventas" sheetId="1" r:id="R61bfbfd76dcb42ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="2" r:id="Rd12e0deebb18480e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="3" r:id="R0e830f3a9026461e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ventas" sheetId="1" r:id="Rda73a2e35b094d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="2" r:id="R59ed771ab3cd43d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="3" r:id="Rcedd0830310a480f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2386,7 +2386,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f58fd653da64012"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf722451490704b21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2524,7 +2524,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae7f76912254f96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R451f02dd25ac4f95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2618,7 +2618,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd09ad67373074f12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7ca74a5193e45b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>